<commit_message>
refactor(templates): retire decision record into tracker, restage docs by dev phase
Retire requirement_decision_record.md: its main table duplicated
requirements_tracker.xlsx ①需求決策 with both hand-maintained (no
generator), violating the one-owner-per-field rule. The tracker is now
the requirement-decision authority: new 核准 approval column on ①,
new ③Gate sheet for milestone sign-off, rationale lives in ②決策沿革.
The /specify hard-gate checklist moves to workflow_manual §8.

Replace Fast/Product/Governed profiles with development stages
(雛型/Pilot/企業級): prototype keeps only tracker skeleton rows + lean
PRD + irreversible-decision ADRs, and the /specify hard gate binds only
from Pilot onward so fuzzy-requirement iteration is not blocked by
approval ceremony. Pilot maps to the 13-doc customer-validation set.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VibeCoding_Workflow_Templates/01_requirements/requirements_tracker.xlsx
+++ b/VibeCoding_Workflow_Templates/01_requirements/requirements_tracker.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="封面" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="① 需求決策" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="② 決策沿革" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="③ Gate" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -519,7 +520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -529,7 +530,7 @@
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
   </cols>
@@ -570,17 +571,22 @@
           <t>狀態</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>核准</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>更新日期</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="K1" s="4" t="inlineStr">
         <is>
           <t>PRD連結</t>
         </is>
@@ -624,20 +630,28 @@
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
+          <t>提案</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
           <t>PM</t>
         </is>
       </c>
-      <c r="I2" s="5" t="inlineStr"/>
-      <c r="J2" s="5" t="inlineStr">
+      <c r="J2" s="5" t="inlineStr"/>
+      <c r="K2" s="5" t="inlineStr">
         <is>
           <t>docs/01_requirements/prd.md</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation sqref="G2:G500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"開放,進行中,Pending,結束,Deferred"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H2:H500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"提案,已核准,延後,取消"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -724,4 +738,109 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Gate ID</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Gate 名稱</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>里程碑</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>前置條件（範圍/驗收）</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>決策</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>決策者</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>日期</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>備註</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>GATE-001</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>（例：M1 需求凍結）</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>（哪些 DEC 已核准）</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>核准</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="n"/>
+      <c r="H2" s="5" t="n"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="E2:E200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"核准,保留,退回"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>